<commit_message>
Add Notion fallback for unattended pipeline runs
- Remove human confirmation prompt after Browse AI parses forward points
  (values are now auto-accepted for unattended operation)
- On Browse AI failure: write today's date to Notion DB and send Gmail
  alert, then abort with recovery instructions
- Add --notion-fallback flag: reads manually-entered bid/ask values from
  Notion and continues the pipeline
- New extract_fwd_points/notion_fallback.py with load_credentials,
  write_failure_code_to_notion, read_forward_points_from_notion,
  send_failure_email helpers
- Update CLAUDE.md with failure flow and recovery instructions
- Include today's master input/output files (2026-03-18)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/swap_implied_input/input_master_1m.xlsx
+++ b/swap_implied_input/input_master_1m.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,6 +514,326 @@
         <v>-25.15</v>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-02-09</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>3.66529</v>
+      </c>
+      <c r="C6" t="n">
+        <v>1.2725</v>
+      </c>
+      <c r="D6" t="n">
+        <v>-25.265</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-02-10</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>3.66529</v>
+      </c>
+      <c r="C7" t="n">
+        <v>1.2668</v>
+      </c>
+      <c r="D7" t="n">
+        <v>-25.25</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-02-11</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>3.66047</v>
+      </c>
+      <c r="C8" t="n">
+        <v>1.2653</v>
+      </c>
+      <c r="D8" t="n">
+        <v>-24.89</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-02-12</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>3.65964</v>
+      </c>
+      <c r="C9" t="n">
+        <v>1.2621</v>
+      </c>
+      <c r="D9" t="n">
+        <v>-25.15</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-02-13</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>3.65964</v>
+      </c>
+      <c r="C10" t="n">
+        <v>1.2621</v>
+      </c>
+      <c r="D10" t="n">
+        <v>-25.255</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-02-14</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>3.65965</v>
+      </c>
+      <c r="C11" t="n">
+        <v>1.2621</v>
+      </c>
+      <c r="D11" t="n">
+        <v>-25.04</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>3.65965</v>
+      </c>
+      <c r="C12" t="n">
+        <v>1.263</v>
+      </c>
+      <c r="D12" t="n">
+        <v>-24.885</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-02-19</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3.66724</v>
+      </c>
+      <c r="C13" t="n">
+        <v>1.266</v>
+      </c>
+      <c r="D13" t="n">
+        <v>-24.33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-02-20</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>3.66724</v>
+      </c>
+      <c r="C14" t="n">
+        <v>1.2686</v>
+      </c>
+      <c r="D14" t="n">
+        <v>-24.345</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-02-24</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>3.67316</v>
+      </c>
+      <c r="C15" t="n">
+        <v>1.2663</v>
+      </c>
+      <c r="D15" t="n">
+        <v>-24.815</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-02-25</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>3.67373</v>
+      </c>
+      <c r="C16" t="n">
+        <v>1.267</v>
+      </c>
+      <c r="D16" t="n">
+        <v>-27.785</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-02-26</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>3.67644</v>
+      </c>
+      <c r="C17" t="n">
+        <v>1.2641</v>
+      </c>
+      <c r="D17" t="n">
+        <v>-27.01</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-02-27</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>3.673</v>
+      </c>
+      <c r="C18" t="n">
+        <v>1.2638</v>
+      </c>
+      <c r="D18" t="n">
+        <v>-27.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-03-10</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>3.66736</v>
+      </c>
+      <c r="C19" t="n">
+        <v>1.282</v>
+      </c>
+      <c r="D19" t="n">
+        <v>-29.665</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3.66996</v>
+      </c>
+      <c r="C20" t="n">
+        <v>1.273</v>
+      </c>
+      <c r="D20" t="n">
+        <v>-28.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-03-12</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>3.67646</v>
+      </c>
+      <c r="C21" t="n">
+        <v>1.273</v>
+      </c>
+      <c r="D21" t="n">
+        <v>-28.56</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-03-13</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>3.67157</v>
+      </c>
+      <c r="C22" t="n">
+        <v>1.2775</v>
+      </c>
+      <c r="D22" t="n">
+        <v>-28.965</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-03-16</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>3.67812</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.2829</v>
+      </c>
+      <c r="D23" t="n">
+        <v>-30.145</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-03-17</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>3.67812</v>
+      </c>
+      <c r="C24" t="n">
+        <v>1.2829</v>
+      </c>
+      <c r="D24" t="n">
+        <v>-29.85</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-03-18</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>3.67956</v>
+      </c>
+      <c r="C25" t="n">
+        <v>1.2769</v>
+      </c>
+      <c r="D25" t="n">
+        <v>-28.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>